<commit_message>
re-render F07 against the re-sorted sweep store it had drifted from
</commit_message>
<xml_diff>
--- a/05_Figures/F07_keepers/c_data/F07_keepers_source_data.xlsx
+++ b/05_Figures/F07_keepers/c_data/F07_keepers_source_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="132">
   <si>
     <t xml:space="preserve">level</t>
   </si>
@@ -55,6 +55,12 @@
     <t xml:space="preserve">null_sd</t>
   </si>
   <si>
+    <t xml:space="preserve">phenotype</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fingerprint</t>
+  </si>
+  <si>
     <t xml:space="preserve">n_screened</t>
   </si>
   <si>
@@ -85,6 +91,12 @@
     <t xml:space="preserve">spls</t>
   </si>
   <si>
+    <t xml:space="preserve">HR_LR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5e6bd8f1d315</t>
+  </si>
+  <si>
     <t xml:space="preserve">pathways|spls|trajectory</t>
   </si>
   <si>
@@ -145,159 +157,174 @@
     <t xml:space="preserve">ridge</t>
   </si>
   <si>
-    <t xml:space="preserve">pathways|ridge|acute</t>
+    <t xml:space="preserve">pathways|ridge|T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ridge  (T1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|plain|T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plain  (T1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|rf|acute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|spls|acute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spls  (acute)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|svm|total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">svm  (total)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|pam|acute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pam  (acute)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|enet|T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enet  (T1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|lasso|T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|ridge|T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proteins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">training</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proteins|svm|training</t>
+  </si>
+  <si>
+    <t xml:space="preserve">svm  (training)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proteins|spls|T2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spls  (T2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proteins|pam|T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pam  (T3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proteins|rf|acute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proteins|enet|T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proteins|lasso|T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proteins|ridge|T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">outcome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spearman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">perm_p_q2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">perm_p_spearman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">null_q2_mean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">null_q2_sd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_1rm_ext</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_mcsa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pathways|enet|trajectory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enet  (trajectory)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comp_hypertrophy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pathways|lasso|trajectory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lasso  (trajectory)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pathways|rf|trajectory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rf  (trajectory)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pathways|ridge|trajectory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ridge  (trajectory)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|lasso|acute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lasso  (acute)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|enet|acute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|spls|trajectory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modules|ridge|acute</t>
   </si>
   <si>
     <t xml:space="preserve">ridge  (acute)</t>
   </si>
   <si>
-    <t xml:space="preserve">modules</t>
-  </si>
-  <si>
-    <t xml:space="preserve">plain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modules|plain|T1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">plain  (T1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modules|rf|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modules|spls|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spls  (acute)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modules|svm|total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">svm  (total)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modules|pam|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pam  (acute)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modules|enet|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modules|lasso|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lasso  (acute)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modules|ridge|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proteins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">training</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proteins|svm|training</t>
-  </si>
-  <si>
-    <t xml:space="preserve">svm  (training)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proteins|spls|T2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spls  (T2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proteins|pam|T3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pam  (T3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proteins|rf|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proteins|enet|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proteins|lasso|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proteins|ridge|acute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">outcome</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spearman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">perm_p_q2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">perm_p_spearman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">null_q2_mean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">null_q2_sd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d_1rm_ext</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d_mcsa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pathways|enet|trajectory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">enet  (trajectory)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">comp_hypertrophy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pathways|lasso|trajectory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lasso  (trajectory)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pathways|rf|trajectory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rf  (trajectory)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pathways|ridge|trajectory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ridge  (trajectory)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modules|spls|trajectory</t>
-  </si>
-  <si>
     <t xml:space="preserve">modules|rf|trajectory</t>
   </si>
   <si>
@@ -332,9 +359,6 @@
   </si>
   <si>
     <t xml:space="preserve">enet  (T2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proteins|lasso|T1</t>
   </si>
   <si>
     <t xml:space="preserve">proteins|ridge|trajectory</t>
@@ -775,16 +799,22 @@
       <c r="T1" t="s">
         <v>19</v>
       </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
         <v>0.729166666666667</v>
@@ -816,37 +846,43 @@
       <c r="M2" t="n">
         <v>0.241947700012745</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+      <c r="O2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P2" t="n">
         <v>7</v>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>0.0625</v>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
         <v>0.875</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>0.5</v>
       </c>
-      <c r="R2" t="b">
-        <v>0</v>
-      </c>
-      <c r="S2" t="s">
-        <v>23</v>
-      </c>
-      <c r="T2" t="s">
-        <v>24</v>
+      <c r="T2" t="b">
+        <v>0</v>
+      </c>
+      <c r="U2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D3" t="n">
         <v>0.660714285714286</v>
@@ -878,37 +914,43 @@
       <c r="M3" t="n">
         <v>0.20099924398478</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" t="n">
         <v>7</v>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>0.0169642857142858</v>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
         <v>0.678571428571429</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
         <v>0.5</v>
       </c>
-      <c r="R3" t="b">
-        <v>0</v>
-      </c>
-      <c r="S3" t="s">
-        <v>27</v>
-      </c>
-      <c r="T3" t="s">
-        <v>28</v>
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
+      <c r="U3" t="s">
+        <v>31</v>
+      </c>
+      <c r="V3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D4" t="n">
         <v>0.446428571428571</v>
@@ -940,37 +982,43 @@
       <c r="M4" t="n">
         <v>0.254413092607442</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+      <c r="O4" t="s">
+        <v>26</v>
+      </c>
+      <c r="P4" t="n">
         <v>7</v>
       </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
         <v>0.786607142857143</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
         <v>0.5</v>
       </c>
-      <c r="R4" t="b">
-        <v>0</v>
-      </c>
-      <c r="S4" t="s">
-        <v>31</v>
-      </c>
-      <c r="T4" t="s">
-        <v>32</v>
+      <c r="T4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U4" t="s">
+        <v>35</v>
+      </c>
+      <c r="V4" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D5" t="n">
         <v>0.4375</v>
@@ -1002,37 +1050,43 @@
       <c r="M5" t="n">
         <v>0.263224498552189</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" t="s">
+        <v>25</v>
+      </c>
+      <c r="O5" t="s">
+        <v>26</v>
+      </c>
+      <c r="P5" t="n">
         <v>7</v>
       </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
         <v>0.751041666666666</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
         <v>0.5</v>
       </c>
-      <c r="R5" t="b">
-        <v>0</v>
-      </c>
-      <c r="S5" t="s">
-        <v>34</v>
-      </c>
-      <c r="T5" t="s">
-        <v>35</v>
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" t="s">
+        <v>38</v>
+      </c>
+      <c r="V5" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D6" t="n">
         <v>0.375</v>
@@ -1064,37 +1118,43 @@
       <c r="M6" t="n">
         <v>0.219723694408278</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" t="s">
+        <v>25</v>
+      </c>
+      <c r="O6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P6" t="n">
         <v>7</v>
       </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
         <v>0.661607142857143</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
         <v>0.5</v>
       </c>
-      <c r="R6" t="b">
-        <v>0</v>
-      </c>
-      <c r="S6" t="s">
-        <v>37</v>
-      </c>
-      <c r="T6" t="s">
-        <v>38</v>
+      <c r="T6" t="b">
+        <v>0</v>
+      </c>
+      <c r="U6" t="s">
+        <v>41</v>
+      </c>
+      <c r="V6" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D7" t="n">
         <v>0.142857142857143</v>
@@ -1126,37 +1186,43 @@
       <c r="M7" t="n">
         <v>0.225962638790841</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P7" t="n">
         <v>7</v>
       </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
         <v>0.6625</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
         <v>0.5</v>
       </c>
-      <c r="R7" t="b">
-        <v>0</v>
-      </c>
-      <c r="S7" t="s">
-        <v>40</v>
-      </c>
-      <c r="T7" t="s">
-        <v>41</v>
+      <c r="T7" t="b">
+        <v>0</v>
+      </c>
+      <c r="U7" t="s">
+        <v>44</v>
+      </c>
+      <c r="V7" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -1183,42 +1249,48 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>0.0158928571428571</v>
+        <v>0.0236607142857143</v>
       </c>
       <c r="M8" t="n">
-        <v>0.090856428083261</v>
-      </c>
-      <c r="N8" t="n">
+        <v>0.100201978811743</v>
+      </c>
+      <c r="N8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O8" t="s">
+        <v>26</v>
+      </c>
+      <c r="P8" t="n">
         <v>7</v>
       </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
       <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.127678571428571</v>
+      </c>
+      <c r="S8" t="n">
         <v>0.5</v>
       </c>
-      <c r="R8" t="b">
-        <v>0</v>
-      </c>
-      <c r="S8" t="s">
-        <v>43</v>
-      </c>
-      <c r="T8" t="s">
-        <v>44</v>
+      <c r="T8" t="b">
+        <v>0</v>
+      </c>
+      <c r="U8" t="s">
+        <v>47</v>
+      </c>
+      <c r="V8" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D9" t="n">
         <v>0.732142857142857</v>
@@ -1250,37 +1322,43 @@
       <c r="M9" t="n">
         <v>0.180024101817027</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" t="n">
         <v>6</v>
       </c>
-      <c r="O9" t="n">
+      <c r="Q9" t="n">
         <v>0.276339285714286</v>
       </c>
-      <c r="P9" t="n">
+      <c r="R9" t="n">
         <v>0.857142857142857</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="S9" t="n">
         <v>0.5</v>
       </c>
-      <c r="R9" t="b">
-        <v>0</v>
-      </c>
-      <c r="S9" t="s">
-        <v>47</v>
-      </c>
-      <c r="T9" t="s">
-        <v>48</v>
+      <c r="T9" t="b">
+        <v>0</v>
+      </c>
+      <c r="U9" t="s">
+        <v>51</v>
+      </c>
+      <c r="V9" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D10" t="n">
         <v>0.5</v>
@@ -1312,37 +1390,43 @@
       <c r="M10" t="n">
         <v>0.203488112035621</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P10" t="n">
         <v>7</v>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>0.0178571428571429</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
         <v>0.696428571428571</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
         <v>0.5</v>
       </c>
-      <c r="R10" t="b">
-        <v>0</v>
-      </c>
-      <c r="S10" t="s">
-        <v>49</v>
-      </c>
-      <c r="T10" t="s">
-        <v>28</v>
+      <c r="T10" t="b">
+        <v>0</v>
+      </c>
+      <c r="U10" t="s">
+        <v>53</v>
+      </c>
+      <c r="V10" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D11" t="n">
         <v>0.5</v>
@@ -1374,37 +1458,43 @@
       <c r="M11" t="n">
         <v>0.213726968807571</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N11" t="s">
+        <v>25</v>
+      </c>
+      <c r="O11" t="s">
+        <v>26</v>
+      </c>
+      <c r="P11" t="n">
         <v>7</v>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>0.0883928571428572</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
         <v>0.767857142857143</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
         <v>0.5</v>
       </c>
-      <c r="R11" t="b">
-        <v>0</v>
-      </c>
-      <c r="S11" t="s">
-        <v>50</v>
-      </c>
-      <c r="T11" t="s">
-        <v>51</v>
+      <c r="T11" t="b">
+        <v>0</v>
+      </c>
+      <c r="U11" t="s">
+        <v>54</v>
+      </c>
+      <c r="V11" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D12" t="n">
         <v>0.375</v>
@@ -1436,37 +1526,43 @@
       <c r="M12" t="n">
         <v>0.25374513246453</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N12" t="s">
+        <v>25</v>
+      </c>
+      <c r="O12" t="s">
+        <v>26</v>
+      </c>
+      <c r="P12" t="n">
         <v>7</v>
       </c>
-      <c r="O12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
         <v>0.791666666666667</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="S12" t="n">
         <v>0.5</v>
       </c>
-      <c r="R12" t="b">
-        <v>0</v>
-      </c>
-      <c r="S12" t="s">
-        <v>53</v>
-      </c>
-      <c r="T12" t="s">
-        <v>54</v>
+      <c r="T12" t="b">
+        <v>0</v>
+      </c>
+      <c r="U12" t="s">
+        <v>57</v>
+      </c>
+      <c r="V12" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D13" t="n">
         <v>0.196428571428571</v>
@@ -1498,37 +1594,43 @@
       <c r="M13" t="n">
         <v>0.181664790036149</v>
       </c>
-      <c r="N13" t="n">
+      <c r="N13" t="s">
+        <v>25</v>
+      </c>
+      <c r="O13" t="s">
+        <v>26</v>
+      </c>
+      <c r="P13" t="n">
         <v>7</v>
       </c>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
         <v>0.517857142857143</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="S13" t="n">
         <v>0.5</v>
       </c>
-      <c r="R13" t="b">
-        <v>0</v>
-      </c>
-      <c r="S13" t="s">
-        <v>55</v>
-      </c>
-      <c r="T13" t="s">
-        <v>56</v>
+      <c r="T13" t="b">
+        <v>0</v>
+      </c>
+      <c r="U13" t="s">
+        <v>59</v>
+      </c>
+      <c r="V13" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -1555,42 +1657,48 @@
         <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>0.0694642857142857</v>
+        <v>0.0658928571428571</v>
       </c>
       <c r="M14" t="n">
-        <v>0.199209335364792</v>
-      </c>
-      <c r="N14" t="n">
+        <v>0.186553391087878</v>
+      </c>
+      <c r="N14" t="s">
+        <v>25</v>
+      </c>
+      <c r="O14" t="s">
+        <v>26</v>
+      </c>
+      <c r="P14" t="n">
         <v>7</v>
       </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0.661607142857143</v>
-      </c>
       <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0.572321428571429</v>
+      </c>
+      <c r="S14" t="n">
         <v>0.5</v>
       </c>
-      <c r="R14" t="b">
-        <v>0</v>
-      </c>
-      <c r="S14" t="s">
-        <v>57</v>
-      </c>
-      <c r="T14" t="s">
-        <v>41</v>
+      <c r="T14" t="b">
+        <v>0</v>
+      </c>
+      <c r="U14" t="s">
+        <v>61</v>
+      </c>
+      <c r="V14" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -1617,42 +1725,48 @@
         <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>0.0728571428571428</v>
+        <v>0.0757142857142857</v>
       </c>
       <c r="M15" t="n">
-        <v>0.216483110032967</v>
-      </c>
-      <c r="N15" t="n">
+        <v>0.206053277165054</v>
+      </c>
+      <c r="N15" t="s">
+        <v>25</v>
+      </c>
+      <c r="O15" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" t="n">
         <v>7</v>
       </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0.733035714285714</v>
-      </c>
       <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.573214285714286</v>
+      </c>
+      <c r="S15" t="n">
         <v>0.5</v>
       </c>
-      <c r="R15" t="b">
-        <v>0</v>
-      </c>
-      <c r="S15" t="s">
-        <v>58</v>
-      </c>
-      <c r="T15" t="s">
-        <v>59</v>
+      <c r="T15" t="b">
+        <v>0</v>
+      </c>
+      <c r="U15" t="s">
+        <v>63</v>
+      </c>
+      <c r="V15" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -1679,42 +1793,48 @@
         <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>0.0238392857142857</v>
+        <v>0.04</v>
       </c>
       <c r="M16" t="n">
-        <v>0.112187953893319</v>
-      </c>
-      <c r="N16" t="n">
+        <v>0.15793582152458</v>
+      </c>
+      <c r="N16" t="s">
+        <v>25</v>
+      </c>
+      <c r="O16" t="s">
+        <v>26</v>
+      </c>
+      <c r="P16" t="n">
         <v>7</v>
       </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0.125892857142857</v>
-      </c>
       <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0.339285714285714</v>
+      </c>
+      <c r="S16" t="n">
         <v>0.5</v>
       </c>
-      <c r="R16" t="b">
-        <v>0</v>
-      </c>
-      <c r="S16" t="s">
-        <v>60</v>
-      </c>
-      <c r="T16" t="s">
-        <v>44</v>
+      <c r="T16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U16" t="s">
+        <v>64</v>
+      </c>
+      <c r="V16" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D17" t="n">
         <v>0.583333333333333</v>
@@ -1746,37 +1866,43 @@
       <c r="M17" t="n">
         <v>0.269594350650839</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N17" t="s">
+        <v>25</v>
+      </c>
+      <c r="O17" t="s">
+        <v>26</v>
+      </c>
+      <c r="P17" t="n">
         <v>7</v>
       </c>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="n">
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
         <v>0.833333333333333</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="S17" t="n">
         <v>0.5</v>
       </c>
-      <c r="R17" t="b">
-        <v>0</v>
-      </c>
-      <c r="S17" t="s">
-        <v>63</v>
-      </c>
-      <c r="T17" t="s">
-        <v>64</v>
+      <c r="T17" t="b">
+        <v>0</v>
+      </c>
+      <c r="U17" t="s">
+        <v>67</v>
+      </c>
+      <c r="V17" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D18" t="n">
         <v>0.535714285714286</v>
@@ -1808,37 +1934,43 @@
       <c r="M18" t="n">
         <v>0.237414669534603</v>
       </c>
-      <c r="N18" t="n">
+      <c r="N18" t="s">
+        <v>25</v>
+      </c>
+      <c r="O18" t="s">
+        <v>26</v>
+      </c>
+      <c r="P18" t="n">
         <v>7</v>
       </c>
-      <c r="O18" t="n">
+      <c r="Q18" t="n">
         <v>0.0705357142857143</v>
       </c>
-      <c r="P18" t="n">
+      <c r="R18" t="n">
         <v>0.840178571428571</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="S18" t="n">
         <v>0.5</v>
       </c>
-      <c r="R18" t="b">
-        <v>0</v>
-      </c>
-      <c r="S18" t="s">
-        <v>66</v>
-      </c>
-      <c r="T18" t="s">
-        <v>67</v>
+      <c r="T18" t="b">
+        <v>0</v>
+      </c>
+      <c r="U18" t="s">
+        <v>70</v>
+      </c>
+      <c r="V18" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B19" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C19" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D19" t="n">
         <v>0.482142857142857</v>
@@ -1870,37 +2002,43 @@
       <c r="M19" t="n">
         <v>0.24394333708367</v>
       </c>
-      <c r="N19" t="n">
+      <c r="N19" t="s">
+        <v>25</v>
+      </c>
+      <c r="O19" t="s">
+        <v>26</v>
+      </c>
+      <c r="P19" t="n">
         <v>7</v>
       </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="n">
         <v>0.715178571428571</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="S19" t="n">
         <v>0.5</v>
       </c>
-      <c r="R19" t="b">
-        <v>0</v>
-      </c>
-      <c r="S19" t="s">
-        <v>69</v>
-      </c>
-      <c r="T19" t="s">
-        <v>70</v>
+      <c r="T19" t="b">
+        <v>0</v>
+      </c>
+      <c r="U19" t="s">
+        <v>73</v>
+      </c>
+      <c r="V19" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D20" t="n">
         <v>0.428571428571428</v>
@@ -1932,37 +2070,43 @@
       <c r="M20" t="n">
         <v>0.19340731063323</v>
       </c>
-      <c r="N20" t="n">
+      <c r="N20" t="s">
+        <v>25</v>
+      </c>
+      <c r="O20" t="s">
+        <v>26</v>
+      </c>
+      <c r="P20" t="n">
         <v>7</v>
       </c>
-      <c r="O20" t="n">
+      <c r="Q20" t="n">
         <v>0.0178571428571429</v>
       </c>
-      <c r="P20" t="n">
+      <c r="R20" t="n">
         <v>0.625892857142857</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="S20" t="n">
         <v>0.5</v>
       </c>
-      <c r="R20" t="b">
-        <v>0</v>
-      </c>
-      <c r="S20" t="s">
-        <v>71</v>
-      </c>
-      <c r="T20" t="s">
-        <v>28</v>
+      <c r="T20" t="b">
+        <v>0</v>
+      </c>
+      <c r="U20" t="s">
+        <v>75</v>
+      </c>
+      <c r="V20" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -1971,7 +2115,7 @@
         <v>15</v>
       </c>
       <c r="F21" t="n">
-        <v>1900</v>
+        <v>1898</v>
       </c>
       <c r="G21" t="n">
         <v>200</v>
@@ -1989,42 +2133,48 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.104196428571429</v>
+        <v>0.1025</v>
       </c>
       <c r="M21" t="n">
-        <v>0.207776661588622</v>
-      </c>
-      <c r="N21" t="n">
+        <v>0.233874073703196</v>
+      </c>
+      <c r="N21" t="s">
+        <v>25</v>
+      </c>
+      <c r="O21" t="s">
+        <v>26</v>
+      </c>
+      <c r="P21" t="n">
         <v>7</v>
       </c>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0.679464285714286</v>
-      </c>
       <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0.734821428571428</v>
+      </c>
+      <c r="S21" t="n">
         <v>0.5</v>
       </c>
-      <c r="R21" t="b">
-        <v>0</v>
-      </c>
-      <c r="S21" t="s">
-        <v>72</v>
-      </c>
-      <c r="T21" t="s">
-        <v>41</v>
+      <c r="T21" t="b">
+        <v>0</v>
+      </c>
+      <c r="U21" t="s">
+        <v>76</v>
+      </c>
+      <c r="V21" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C22" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -2033,7 +2183,7 @@
         <v>15</v>
       </c>
       <c r="F22" t="n">
-        <v>1900</v>
+        <v>1898</v>
       </c>
       <c r="G22" t="n">
         <v>200</v>
@@ -2051,42 +2201,48 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>0.113214285714286</v>
+        <v>0.105625</v>
       </c>
       <c r="M22" t="n">
-        <v>0.213674949161307</v>
-      </c>
-      <c r="N22" t="n">
+        <v>0.235543575607896</v>
+      </c>
+      <c r="N22" t="s">
+        <v>25</v>
+      </c>
+      <c r="O22" t="s">
+        <v>26</v>
+      </c>
+      <c r="P22" t="n">
         <v>7</v>
       </c>
-      <c r="O22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" t="n">
-        <v>0.591964285714284</v>
-      </c>
       <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.734821428571428</v>
+      </c>
+      <c r="S22" t="n">
         <v>0.5</v>
       </c>
-      <c r="R22" t="b">
-        <v>0</v>
-      </c>
-      <c r="S22" t="s">
-        <v>73</v>
-      </c>
-      <c r="T22" t="s">
-        <v>59</v>
+      <c r="T22" t="b">
+        <v>0</v>
+      </c>
+      <c r="U22" t="s">
+        <v>77</v>
+      </c>
+      <c r="V22" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B23" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C23" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -2095,7 +2251,7 @@
         <v>15</v>
       </c>
       <c r="F23" t="n">
-        <v>1900</v>
+        <v>1898</v>
       </c>
       <c r="G23" t="n">
         <v>200</v>
@@ -2113,31 +2269,37 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0.00205357142857143</v>
+        <v>0.035625</v>
       </c>
       <c r="M23" t="n">
-        <v>0.0266238528978017</v>
-      </c>
-      <c r="N23" t="n">
+        <v>0.142402109792109</v>
+      </c>
+      <c r="N23" t="s">
+        <v>25</v>
+      </c>
+      <c r="O23" t="s">
+        <v>26</v>
+      </c>
+      <c r="P23" t="n">
         <v>7</v>
       </c>
-      <c r="O23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0</v>
-      </c>
       <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.429464285714286</v>
+      </c>
+      <c r="S23" t="n">
         <v>0.5</v>
       </c>
-      <c r="R23" t="b">
-        <v>0</v>
-      </c>
-      <c r="S23" t="s">
-        <v>74</v>
-      </c>
-      <c r="T23" t="s">
-        <v>44</v>
+      <c r="T23" t="b">
+        <v>0</v>
+      </c>
+      <c r="U23" t="s">
+        <v>78</v>
+      </c>
+      <c r="V23" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2159,7 +2321,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -2174,40 +2336,40 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="J1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="K1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="L1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="M1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
         <v>3</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>10</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
         <v>12</v>
-      </c>
-      <c r="R1" t="s">
-        <v>13</v>
-      </c>
-      <c r="S1" t="s">
-        <v>14</v>
       </c>
       <c r="T1" t="s">
         <v>15</v>
@@ -2224,19 +2386,25 @@
       <c r="X1" t="s">
         <v>19</v>
       </c>
+      <c r="Y1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E2" t="n">
         <v>14</v>
@@ -2265,52 +2433,58 @@
       <c r="M2" t="n">
         <v>0.958346038400894</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" t="s">
+        <v>86</v>
+      </c>
+      <c r="O2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P2" t="n">
         <v>0.620937211013559</v>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>0.00497512437810945</v>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
         <v>-1.01739479271618</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>0.958346038400894</v>
       </c>
-      <c r="R2" t="n">
+      <c r="T2" t="n">
         <v>42</v>
       </c>
-      <c r="S2" t="n">
+      <c r="U2" t="n">
         <v>-2.99597796957357</v>
       </c>
-      <c r="T2" t="n">
+      <c r="V2" t="n">
         <v>0.213535024255417</v>
       </c>
-      <c r="U2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" t="b">
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="b">
         <v>1</v>
       </c>
-      <c r="W2" t="s">
-        <v>31</v>
-      </c>
-      <c r="X2" t="s">
-        <v>32</v>
+      <c r="Y2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E3" t="n">
         <v>14</v>
@@ -2339,52 +2513,58 @@
       <c r="M3" t="n">
         <v>0.731814620750024</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" t="s">
+        <v>87</v>
+      </c>
+      <c r="O3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" t="n">
         <v>0.411266403925074</v>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>0.0298507462686567</v>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
         <v>-0.746450270442581</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
         <v>0.731814620750024</v>
       </c>
-      <c r="R3" t="n">
+      <c r="T3" t="n">
         <v>42</v>
       </c>
-      <c r="S3" t="n">
+      <c r="U3" t="n">
         <v>-2.19270612623952</v>
       </c>
-      <c r="T3" t="n">
+      <c r="V3" t="n">
         <v>0.296474501089059</v>
       </c>
-      <c r="U3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" t="b">
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="b">
         <v>1</v>
       </c>
-      <c r="W3" t="s">
-        <v>23</v>
-      </c>
-      <c r="X3" t="s">
-        <v>24</v>
+      <c r="Y3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E4" t="n">
         <v>14</v>
@@ -2413,52 +2593,58 @@
       <c r="M4" t="n">
         <v>0.138191298603544</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" t="s">
+        <v>87</v>
+      </c>
+      <c r="O4" t="s">
+        <v>26</v>
+      </c>
+      <c r="P4" t="n">
         <v>0.259726105892755</v>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>0.0248756218905473</v>
       </c>
-      <c r="P4" t="n">
+      <c r="R4" t="n">
         <v>-0.186438934688261</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
         <v>0.138191298603544</v>
       </c>
-      <c r="R4" t="n">
+      <c r="T4" t="n">
         <v>42</v>
       </c>
-      <c r="S4" t="n">
+      <c r="U4" t="n">
         <v>-0.378679567874654</v>
       </c>
-      <c r="T4" t="n">
+      <c r="V4" t="n">
         <v>0.0423994795376123</v>
       </c>
-      <c r="U4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" t="b">
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="b">
         <v>1</v>
       </c>
-      <c r="W4" t="s">
-        <v>84</v>
-      </c>
-      <c r="X4" t="s">
-        <v>85</v>
+      <c r="Y4" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E5" t="n">
         <v>14</v>
@@ -2487,52 +2673,58 @@
       <c r="M5" t="n">
         <v>0.192339074737823</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" t="s">
+        <v>90</v>
+      </c>
+      <c r="O5" t="s">
+        <v>26</v>
+      </c>
+      <c r="P5" t="n">
         <v>0.17778999080829</v>
       </c>
-      <c r="O5" t="n">
+      <c r="Q5" t="n">
         <v>0.0348258706467662</v>
       </c>
-      <c r="P5" t="n">
+      <c r="R5" t="n">
         <v>-0.212031969926516</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
         <v>0.192339074737823</v>
       </c>
-      <c r="R5" t="n">
+      <c r="T5" t="n">
         <v>42</v>
       </c>
-      <c r="S5" t="n">
+      <c r="U5" t="n">
         <v>-0.483899319109462</v>
       </c>
-      <c r="T5" t="n">
+      <c r="V5" t="n">
         <v>0.0605621809575338</v>
       </c>
-      <c r="U5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" t="b">
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="b">
         <v>1</v>
       </c>
-      <c r="W5" t="s">
-        <v>87</v>
-      </c>
-      <c r="X5" t="s">
-        <v>88</v>
+      <c r="Y5" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E6" t="n">
         <v>14</v>
@@ -2561,52 +2753,58 @@
       <c r="M6" t="n">
         <v>0.136850848173076</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" t="s">
+        <v>87</v>
+      </c>
+      <c r="O6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P6" t="n">
         <v>0.162702655113724</v>
       </c>
-      <c r="O6" t="n">
+      <c r="Q6" t="n">
         <v>0.0199004975124378</v>
       </c>
-      <c r="P6" t="n">
+      <c r="R6" t="n">
         <v>-0.192847165091876</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
         <v>0.136850848173076</v>
       </c>
-      <c r="R6" t="n">
+      <c r="T6" t="n">
         <v>42</v>
       </c>
-      <c r="S6" t="n">
+      <c r="U6" t="n">
         <v>-0.388055651191463</v>
       </c>
-      <c r="T6" t="n">
+      <c r="V6" t="n">
         <v>0.0565154017031282</v>
       </c>
-      <c r="U6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" t="b">
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="b">
         <v>1</v>
       </c>
-      <c r="W6" t="s">
-        <v>89</v>
-      </c>
-      <c r="X6" t="s">
-        <v>90</v>
+      <c r="Y6" t="s">
+        <v>93</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E7" t="n">
         <v>14</v>
@@ -2635,52 +2833,58 @@
       <c r="M7" t="n">
         <v>0.0457359998087378</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" t="s">
+        <v>87</v>
+      </c>
+      <c r="O7" t="s">
+        <v>26</v>
+      </c>
+      <c r="P7" t="n">
         <v>0.077556765871716</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>0.0099502487562189</v>
       </c>
-      <c r="P7" t="n">
+      <c r="R7" t="n">
         <v>-0.157106296210139</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
         <v>0.0457359998087378</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>42</v>
       </c>
-      <c r="S7" t="n">
+      <c r="U7" t="n">
         <v>-0.193426444665325</v>
       </c>
-      <c r="T7" t="n">
+      <c r="V7" t="n">
         <v>-0.119187208873766</v>
       </c>
-      <c r="U7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" t="b">
+      <c r="W7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" t="b">
         <v>1</v>
       </c>
-      <c r="W7" t="s">
-        <v>91</v>
-      </c>
-      <c r="X7" t="s">
-        <v>92</v>
+      <c r="Y7" t="s">
+        <v>95</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E8" t="n">
         <v>15</v>
@@ -2709,52 +2913,58 @@
       <c r="M8" t="n">
         <v>1.04103533694376</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N8" t="s">
+        <v>87</v>
+      </c>
+      <c r="O8" t="s">
+        <v>26</v>
+      </c>
+      <c r="P8" t="n">
         <v>0.462372213177816</v>
       </c>
-      <c r="O8" t="n">
+      <c r="Q8" t="n">
         <v>0.0199004975124378</v>
       </c>
-      <c r="P8" t="n">
+      <c r="R8" t="n">
         <v>-0.452720615773047</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="S8" t="n">
         <v>1.04103533694376</v>
       </c>
-      <c r="R8" t="n">
+      <c r="T8" t="n">
         <v>42</v>
       </c>
-      <c r="S8" t="n">
+      <c r="U8" t="n">
         <v>-1.71279244365411</v>
       </c>
-      <c r="T8" t="n">
+      <c r="V8" t="n">
         <v>-0.0859061716097375</v>
       </c>
-      <c r="U8" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" t="b">
+      <c r="W8" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" t="b">
         <v>1</v>
       </c>
-      <c r="W8" t="s">
-        <v>58</v>
-      </c>
-      <c r="X8" t="s">
-        <v>59</v>
+      <c r="Y8" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E9" t="n">
         <v>15</v>
@@ -2783,52 +2993,58 @@
       <c r="M9" t="n">
         <v>1.06810987167105</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" t="s">
+        <v>87</v>
+      </c>
+      <c r="O9" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" t="n">
         <v>0.444504844977317</v>
       </c>
-      <c r="O9" t="n">
+      <c r="Q9" t="n">
         <v>0.0199004975124378</v>
       </c>
-      <c r="P9" t="n">
+      <c r="R9" t="n">
         <v>-0.453419917090597</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="S9" t="n">
         <v>1.06810987167105</v>
       </c>
-      <c r="R9" t="n">
+      <c r="T9" t="n">
         <v>42</v>
       </c>
-      <c r="S9" t="n">
+      <c r="U9" t="n">
         <v>-1.73254734585726</v>
       </c>
-      <c r="T9" t="n">
+      <c r="V9" t="n">
         <v>-0.00254606388241447</v>
       </c>
-      <c r="U9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" t="b">
+      <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="b">
         <v>1</v>
       </c>
-      <c r="W9" t="s">
-        <v>57</v>
-      </c>
-      <c r="X9" t="s">
-        <v>41</v>
+      <c r="Y9" t="s">
+        <v>99</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E10" t="n">
         <v>14</v>
@@ -2857,52 +3073,58 @@
       <c r="M10" t="n">
         <v>0.667080536893519</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N10" t="s">
+        <v>87</v>
+      </c>
+      <c r="O10" t="s">
+        <v>26</v>
+      </c>
+      <c r="P10" t="n">
         <v>0.400204457349602</v>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>0.0149253731343284</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
         <v>-0.631937274941917</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
         <v>0.667080536893519</v>
       </c>
-      <c r="R10" t="n">
+      <c r="T10" t="n">
         <v>42</v>
       </c>
-      <c r="S10" t="n">
+      <c r="U10" t="n">
         <v>-1.73878951444609</v>
       </c>
-      <c r="T10" t="n">
+      <c r="V10" t="n">
         <v>0.194239379625306</v>
       </c>
-      <c r="U10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V10" t="b">
+      <c r="W10" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" t="b">
         <v>1</v>
       </c>
-      <c r="W10" t="s">
-        <v>93</v>
-      </c>
-      <c r="X10" t="s">
-        <v>24</v>
+      <c r="Y10" t="s">
+        <v>100</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E11" t="n">
         <v>15</v>
@@ -2931,52 +3153,58 @@
       <c r="M11" t="n">
         <v>0.150327693860948</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N11" t="s">
+        <v>87</v>
+      </c>
+      <c r="O11" t="s">
+        <v>26</v>
+      </c>
+      <c r="P11" t="n">
         <v>0.395420724337231</v>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>0.0149253731343284</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
         <v>-0.173624781822918</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
         <v>0.150327693860948</v>
       </c>
-      <c r="R11" t="n">
+      <c r="T11" t="n">
         <v>42</v>
       </c>
-      <c r="S11" t="n">
+      <c r="U11" t="n">
         <v>-0.386875093221916</v>
       </c>
-      <c r="T11" t="n">
+      <c r="V11" t="n">
         <v>-0.00285242014711681</v>
       </c>
-      <c r="U11" t="n">
-        <v>0</v>
-      </c>
-      <c r="V11" t="b">
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="b">
         <v>1</v>
       </c>
-      <c r="W11" t="s">
-        <v>60</v>
-      </c>
-      <c r="X11" t="s">
-        <v>44</v>
+      <c r="Y11" t="s">
+        <v>101</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E12" t="n">
         <v>14</v>
@@ -3005,52 +3233,58 @@
       <c r="M12" t="n">
         <v>0.875160051717567</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N12" t="s">
+        <v>87</v>
+      </c>
+      <c r="O12" t="s">
+        <v>26</v>
+      </c>
+      <c r="P12" t="n">
         <v>0.392983399454889</v>
       </c>
-      <c r="O12" t="n">
+      <c r="Q12" t="n">
         <v>0.0248756218905473</v>
       </c>
-      <c r="P12" t="n">
+      <c r="R12" t="n">
         <v>-1.07563199840268</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="S12" t="n">
         <v>0.875160051717567</v>
       </c>
-      <c r="R12" t="n">
+      <c r="T12" t="n">
         <v>42</v>
       </c>
-      <c r="S12" t="n">
+      <c r="U12" t="n">
         <v>-2.44133225480704</v>
       </c>
-      <c r="T12" t="n">
+      <c r="V12" t="n">
         <v>0.157076548920688</v>
       </c>
-      <c r="U12" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" t="b">
+      <c r="W12" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" t="b">
         <v>1</v>
       </c>
-      <c r="W12" t="s">
-        <v>53</v>
-      </c>
-      <c r="X12" t="s">
-        <v>54</v>
+      <c r="Y12" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D13" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E13" t="n">
         <v>14</v>
@@ -3079,52 +3313,58 @@
       <c r="M13" t="n">
         <v>0.176778018485117</v>
       </c>
-      <c r="N13" t="n">
+      <c r="N13" t="s">
+        <v>87</v>
+      </c>
+      <c r="O13" t="s">
+        <v>26</v>
+      </c>
+      <c r="P13" t="n">
         <v>0.37156217891133</v>
       </c>
-      <c r="O13" t="n">
+      <c r="Q13" t="n">
         <v>0.00497512437810945</v>
       </c>
-      <c r="P13" t="n">
+      <c r="R13" t="n">
         <v>-0.225358543648482</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="S13" t="n">
         <v>0.176778018485117</v>
       </c>
-      <c r="R13" t="n">
+      <c r="T13" t="n">
         <v>42</v>
       </c>
-      <c r="S13" t="n">
+      <c r="U13" t="n">
         <v>-0.524493540079265</v>
       </c>
-      <c r="T13" t="n">
+      <c r="V13" t="n">
         <v>0.072643159223403</v>
       </c>
-      <c r="U13" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" t="b">
+      <c r="W13" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" t="b">
         <v>1</v>
       </c>
-      <c r="W13" t="s">
+      <c r="Y13" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z13" t="s">
         <v>94</v>
-      </c>
-      <c r="X13" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C14" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D14" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E14" t="n">
         <v>15</v>
@@ -3153,52 +3393,58 @@
       <c r="M14" t="n">
         <v>104.537681598421</v>
       </c>
-      <c r="N14" t="n">
+      <c r="N14" t="s">
+        <v>87</v>
+      </c>
+      <c r="O14" t="s">
+        <v>26</v>
+      </c>
+      <c r="P14" t="n">
         <v>0.140992211958394</v>
       </c>
-      <c r="O14" t="n">
+      <c r="Q14" t="n">
         <v>0.0149253731343284</v>
       </c>
-      <c r="P14" t="n">
+      <c r="R14" t="n">
         <v>-93.540728185107</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="S14" t="n">
         <v>104.537681598421</v>
       </c>
-      <c r="R14" t="n">
+      <c r="T14" t="n">
         <v>36</v>
       </c>
-      <c r="S14" t="n">
+      <c r="U14" t="n">
         <v>-268.301815756177</v>
       </c>
-      <c r="T14" t="n">
+      <c r="V14" t="n">
         <v>-2.6774278902307</v>
       </c>
-      <c r="U14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" t="b">
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="b">
         <v>1</v>
       </c>
-      <c r="W14" t="s">
-        <v>95</v>
-      </c>
-      <c r="X14" t="s">
-        <v>96</v>
+      <c r="Y14" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E15" t="n">
         <v>15</v>
@@ -3227,52 +3473,58 @@
       <c r="M15" t="n">
         <v>0.667080858461555</v>
       </c>
-      <c r="N15" t="n">
+      <c r="N15" t="s">
+        <v>106</v>
+      </c>
+      <c r="O15" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" t="n">
         <v>0.457722008481763</v>
       </c>
-      <c r="O15" t="n">
+      <c r="Q15" t="n">
         <v>0.0298507462686567</v>
       </c>
-      <c r="P15" t="n">
+      <c r="R15" t="n">
         <v>-0.728741920372084</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="S15" t="n">
         <v>0.667080858461555</v>
       </c>
-      <c r="R15" t="n">
+      <c r="T15" t="n">
         <v>42</v>
       </c>
-      <c r="S15" t="n">
+      <c r="U15" t="n">
         <v>-1.82463181426028</v>
       </c>
-      <c r="T15" t="n">
+      <c r="V15" t="n">
         <v>0.30510650070914</v>
       </c>
-      <c r="U15" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" t="b">
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="b">
         <v>1</v>
       </c>
-      <c r="W15" t="s">
-        <v>98</v>
-      </c>
-      <c r="X15" t="s">
-        <v>99</v>
+      <c r="Y15" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D16" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E16" t="n">
         <v>15</v>
@@ -3301,52 +3553,58 @@
       <c r="M16" t="n">
         <v>0.325815812872284</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N16" t="s">
+        <v>87</v>
+      </c>
+      <c r="O16" t="s">
+        <v>26</v>
+      </c>
+      <c r="P16" t="n">
         <v>0.355394439064757</v>
       </c>
-      <c r="O16" t="n">
+      <c r="Q16" t="n">
         <v>0.0248756218905473</v>
       </c>
-      <c r="P16" t="n">
+      <c r="R16" t="n">
         <v>-0.354732305755251</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="S16" t="n">
         <v>0.325815812872284</v>
       </c>
-      <c r="R16" t="n">
+      <c r="T16" t="n">
         <v>42</v>
       </c>
-      <c r="S16" t="n">
+      <c r="U16" t="n">
         <v>-0.849998638044073</v>
       </c>
-      <c r="T16" t="n">
+      <c r="V16" t="n">
         <v>0.150065426610544</v>
       </c>
-      <c r="U16" t="n">
-        <v>0</v>
-      </c>
-      <c r="V16" t="b">
+      <c r="W16" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" t="b">
         <v>1</v>
       </c>
-      <c r="W16" t="s">
-        <v>100</v>
-      </c>
-      <c r="X16" t="s">
-        <v>101</v>
+      <c r="Y16" t="s">
+        <v>109</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D17" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E17" t="n">
         <v>15</v>
@@ -3375,52 +3633,58 @@
       <c r="M17" t="n">
         <v>0.128940063668492</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N17" t="s">
+        <v>87</v>
+      </c>
+      <c r="O17" t="s">
+        <v>26</v>
+      </c>
+      <c r="P17" t="n">
         <v>0.0866834108093932</v>
       </c>
-      <c r="O17" t="n">
+      <c r="Q17" t="n">
         <v>0.0348258706467662</v>
       </c>
-      <c r="P17" t="n">
+      <c r="R17" t="n">
         <v>-0.170939231628711</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="S17" t="n">
         <v>0.128940063668492</v>
       </c>
-      <c r="R17" t="n">
+      <c r="T17" t="n">
         <v>42</v>
       </c>
-      <c r="S17" t="n">
+      <c r="U17" t="n">
         <v>-0.366143996644589</v>
       </c>
-      <c r="T17" t="n">
+      <c r="V17" t="n">
         <v>0.043195208363013</v>
       </c>
-      <c r="U17" t="n">
-        <v>0</v>
-      </c>
-      <c r="V17" t="b">
+      <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="b">
         <v>1</v>
       </c>
-      <c r="W17" t="s">
-        <v>102</v>
-      </c>
-      <c r="X17" t="s">
-        <v>103</v>
+      <c r="Y17" t="s">
+        <v>111</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D18" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E18" t="n">
         <v>15</v>
@@ -3449,52 +3713,58 @@
       <c r="M18" t="n">
         <v>0.0916940773108943</v>
       </c>
-      <c r="N18" t="n">
+      <c r="N18" t="s">
+        <v>87</v>
+      </c>
+      <c r="O18" t="s">
+        <v>26</v>
+      </c>
+      <c r="P18" t="n">
         <v>0.0365935847765777</v>
       </c>
-      <c r="O18" t="n">
+      <c r="Q18" t="n">
         <v>0.0398009950248756</v>
       </c>
-      <c r="P18" t="n">
+      <c r="R18" t="n">
         <v>-0.150062832444744</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="S18" t="n">
         <v>0.0916940773108943</v>
       </c>
-      <c r="R18" t="n">
+      <c r="T18" t="n">
         <v>42</v>
       </c>
-      <c r="S18" t="n">
+      <c r="U18" t="n">
         <v>-0.250226196917061</v>
       </c>
-      <c r="T18" t="n">
+      <c r="V18" t="n">
         <v>-0.0440590134715418</v>
       </c>
-      <c r="U18" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" t="b">
+      <c r="W18" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" t="b">
         <v>1</v>
       </c>
-      <c r="W18" t="s">
-        <v>104</v>
-      </c>
-      <c r="X18" t="s">
-        <v>105</v>
+      <c r="Y18" t="s">
+        <v>113</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B19" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C19" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D19" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E19" t="n">
         <v>15</v>
@@ -3523,52 +3793,58 @@
       <c r="M19" t="n">
         <v>0.145788357211688</v>
       </c>
-      <c r="N19" t="n">
+      <c r="N19" t="s">
+        <v>106</v>
+      </c>
+      <c r="O19" t="s">
+        <v>26</v>
+      </c>
+      <c r="P19" t="n">
         <v>-0.0210078015160711</v>
       </c>
-      <c r="O19" t="n">
+      <c r="Q19" t="n">
         <v>0.0895522388059701</v>
       </c>
-      <c r="P19" t="n">
+      <c r="R19" t="n">
         <v>-0.17561000952502</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="S19" t="n">
         <v>0.145788357211688</v>
       </c>
-      <c r="R19" t="n">
+      <c r="T19" t="n">
         <v>42</v>
       </c>
-      <c r="S19" t="n">
+      <c r="U19" t="n">
         <v>-0.393686497706517</v>
       </c>
-      <c r="T19" t="n">
+      <c r="V19" t="n">
         <v>0.0752378579364235</v>
       </c>
-      <c r="U19" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" t="b">
-        <v>0</v>
-      </c>
-      <c r="W19" t="s">
-        <v>106</v>
-      </c>
-      <c r="X19" t="s">
-        <v>38</v>
+      <c r="W19" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>77</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E20" t="n">
         <v>14</v>
@@ -3597,38 +3873,44 @@
       <c r="M20" t="n">
         <v>0.0235080662093789</v>
       </c>
-      <c r="N20" t="n">
+      <c r="N20" t="s">
+        <v>87</v>
+      </c>
+      <c r="O20" t="s">
+        <v>26</v>
+      </c>
+      <c r="P20" t="n">
         <v>-0.0256414156241849</v>
       </c>
-      <c r="O20" t="n">
+      <c r="Q20" t="n">
         <v>0.0099502487562189</v>
       </c>
-      <c r="P20" t="n">
+      <c r="R20" t="n">
         <v>-0.160664435323007</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="S20" t="n">
         <v>0.0235080662093789</v>
       </c>
-      <c r="R20" t="n">
+      <c r="T20" t="n">
         <v>42</v>
       </c>
-      <c r="S20" t="n">
+      <c r="U20" t="n">
         <v>-0.184320257891312</v>
       </c>
-      <c r="T20" t="n">
+      <c r="V20" t="n">
         <v>-0.159763313609467</v>
       </c>
-      <c r="U20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" t="b">
-        <v>0</v>
-      </c>
-      <c r="W20" t="s">
-        <v>107</v>
-      </c>
-      <c r="X20" t="s">
-        <v>92</v>
+      <c r="W20" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>115</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -3644,24 +3926,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B1" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B2" t="n">
         <v>0.24634128468443</v>
@@ -3670,15 +3952,15 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="B3" t="n">
         <v>0.595923521891115</v>
@@ -3687,15 +3969,15 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E3" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B4" t="n">
         <v>0.0714725596606504</v>
@@ -3704,15 +3986,15 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E4" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B5" t="n">
         <v>0.106296359589286</v>
@@ -3721,15 +4003,15 @@
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E5" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B6" t="n">
         <v>0.996331871821693</v>
@@ -3738,15 +4020,15 @@
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E6" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B7" t="n">
         <v>0.70749566734604</v>
@@ -3755,15 +4037,15 @@
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E7" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B8" t="n">
         <v>0.452009408018053</v>
@@ -3772,15 +4054,15 @@
         <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E8" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B9" t="n">
         <v>0.93828696756471</v>
@@ -3789,15 +4071,15 @@
         <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E9" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B10" t="n">
         <v>0.790766933331937</v>
@@ -3806,15 +4088,15 @@
         <v>0</v>
       </c>
       <c r="D10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E10" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B11" t="n">
         <v>0.860463045375293</v>
@@ -3823,15 +4105,15 @@
         <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="B12" t="n">
         <v>0.976623637038833</v>
@@ -3840,15 +4122,15 @@
         <v>0</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B13" t="n">
         <v>0.0372181644372705</v>
@@ -3857,15 +4139,15 @@
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B14" t="n">
         <v>0.00111117207844174</v>
@@ -3874,15 +4156,15 @@
         <v>3</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B15" t="n">
         <v>0.925486027942554</v>
@@ -3891,15 +4173,15 @@
         <v>0</v>
       </c>
       <c r="D15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B16" t="n">
         <v>0.96180441127636</v>
@@ -3908,15 +4190,15 @@
         <v>0</v>
       </c>
       <c r="D16" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B17" t="n">
         <v>0.133517708139971</v>
@@ -3925,15 +4207,15 @@
         <v>0</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B18" t="n">
         <v>0.822899730107993</v>
@@ -3942,15 +4224,15 @@
         <v>0</v>
       </c>
       <c r="D18" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B19" t="n">
         <v>0.0425029672208257</v>
@@ -3959,15 +4241,15 @@
         <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B20" t="n">
         <v>0.241186637828355</v>
@@ -3976,15 +4258,15 @@
         <v>0</v>
       </c>
       <c r="D20" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E20" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="B21" t="n">
         <v>0.941846637807116</v>
@@ -3993,15 +4275,15 @@
         <v>0</v>
       </c>
       <c r="D21" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E21" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B22" t="n">
         <v>0.0823720753199149</v>
@@ -4010,15 +4292,15 @@
         <v>0</v>
       </c>
       <c r="D22" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B23" t="n">
         <v>0.527193126890309</v>
@@ -4027,15 +4309,15 @@
         <v>0</v>
       </c>
       <c r="D23" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E23" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B24" t="n">
         <v>0.922584841692793</v>
@@ -4044,15 +4326,15 @@
         <v>0</v>
       </c>
       <c r="D24" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E24" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B25" t="n">
         <v>0.876530916682701</v>
@@ -4061,15 +4343,15 @@
         <v>0</v>
       </c>
       <c r="D25" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E25" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B26" t="n">
         <v>0.384311055119259</v>
@@ -4078,15 +4360,15 @@
         <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E26" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B27" t="n">
         <v>0.708162829885467</v>
@@ -4095,15 +4377,15 @@
         <v>0</v>
       </c>
       <c r="D27" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E27" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B28" t="n">
         <v>0.418656058555944</v>
@@ -4112,10 +4394,10 @@
         <v>0</v>
       </c>
       <c r="D28" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>